<commit_message>
Update player master files 31/03/26
</commit_message>
<xml_diff>
--- a/data/players/James_Plant_master.xlsx
+++ b/data/players/James_Plant_master.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Physical" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressing" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Off_Ball_Runs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match_by_Match" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wyscout" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Physical" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pressing" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Off_Ball_Runs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Match_by_Match" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Wyscout" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Merged" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,10 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -62,12 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -766,15 +763,18 @@
       <c r="AH2" t="n">
         <v>0.71</v>
       </c>
+      <c r="AI2" t="inlineStr"/>
       <c r="AJ2" t="n">
         <v>2</v>
       </c>
       <c r="AK2" t="n">
         <v>1.63</v>
       </c>
+      <c r="AL2" t="inlineStr"/>
       <c r="AM2" t="n">
         <v>11</v>
       </c>
+      <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="n">
         <v>3.1</v>
       </c>
@@ -908,6 +908,8 @@
       <c r="AJ3" t="n">
         <v>0</v>
       </c>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
       <c r="AM3" t="n">
         <v>38</v>
       </c>
@@ -1041,9 +1043,12 @@
       <c r="AH4" t="n">
         <v>0.6899999999999999</v>
       </c>
+      <c r="AI4" t="inlineStr"/>
       <c r="AJ4" t="n">
         <v>0</v>
       </c>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="n">
         <v>55</v>
       </c>
@@ -1177,9 +1182,12 @@
       <c r="AH5" t="n">
         <v>0.74</v>
       </c>
+      <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="n">
         <v>0</v>
       </c>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
       <c r="AM5" t="n">
         <v>53</v>
       </c>
@@ -1322,6 +1330,7 @@
       <c r="AK6" t="n">
         <v>2.03</v>
       </c>
+      <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="n">
         <v>34</v>
       </c>
@@ -1597,9 +1606,13 @@
       <c r="AG8" t="n">
         <v>0</v>
       </c>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="n">
         <v>0</v>
       </c>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
       <c r="AM8" t="n">
         <v>54</v>
       </c>
@@ -1730,9 +1743,13 @@
       <c r="AG9" t="n">
         <v>0</v>
       </c>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
       <c r="AJ9" t="n">
         <v>0</v>
       </c>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
       <c r="AM9" t="n">
         <v>11</v>
       </c>
@@ -1872,6 +1889,8 @@
       <c r="AJ10" t="n">
         <v>0</v>
       </c>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
       <c r="AM10" t="n">
         <v>41</v>
       </c>
@@ -2211,12 +2230,14 @@
       <c r="AG2" t="n">
         <v>0</v>
       </c>
+      <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" t="n">
         <v>0</v>
       </c>
+      <c r="AK2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -3653,12 +3674,18 @@
       <c r="AA2" t="n">
         <v>5</v>
       </c>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="n">
         <v>2</v>
       </c>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="n">
         <v>11</v>
       </c>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3750,12 +3777,18 @@
       <c r="AA3" t="n">
         <v>3</v>
       </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="n">
         <v>0</v>
       </c>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="n">
         <v>38</v>
       </c>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3847,12 +3880,18 @@
       <c r="AA4" t="n">
         <v>7</v>
       </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="n">
         <v>0</v>
       </c>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="n">
         <v>55</v>
       </c>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3944,12 +3983,18 @@
       <c r="AA5" t="n">
         <v>5</v>
       </c>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="n">
         <v>0</v>
       </c>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="n">
         <v>53</v>
       </c>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4041,12 +4086,18 @@
       <c r="AA6" t="n">
         <v>3</v>
       </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="n">
         <v>2</v>
       </c>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="n">
         <v>34</v>
       </c>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4138,12 +4189,18 @@
       <c r="AA7" t="n">
         <v>4</v>
       </c>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="n">
         <v>2</v>
       </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="n">
         <v>40</v>
       </c>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4178,12 +4235,37 @@
       <c r="H8" t="n">
         <v>1214</v>
       </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
       </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr"/>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4275,12 +4357,18 @@
       <c r="AA9" t="n">
         <v>0</v>
       </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="n">
         <v>0</v>
       </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="n">
         <v>54</v>
       </c>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4372,12 +4460,18 @@
       <c r="AA10" t="n">
         <v>0</v>
       </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="n">
         <v>0</v>
       </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="n">
         <v>11</v>
       </c>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4469,12 +4563,18 @@
       <c r="AA11" t="n">
         <v>4</v>
       </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="n">
         <v>0</v>
       </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="n">
         <v>41</v>
       </c>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4491,362 +4591,362 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Match</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Competition</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Minutes played</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Total actions</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>successful</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Goals</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Assists</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Shots</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>on target</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>xG</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Passes</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>accurate passes</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Long passes</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>accurate long passes</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Crosses</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>accurate crosses</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Dribbles</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>successful dribbles</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>successful</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Duels</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>won</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Aerial duels</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>won.1</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>won</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Interceptions</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Losses</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>own half</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Recoveries</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>opp. half</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Yellow card</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Red card</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Defensive duels</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>won.2</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>Loose ball duels / won</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>Unnamed: 34</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>Sliding tackles / successful</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>Unnamed: 36</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>won</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Loose ball duels</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>won</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Sliding tackles</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>successful</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Clearances</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Fouls</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Yellow cards</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Red cards</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Shot assists</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Offensive duels</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
-        <is>
-          <t>won.4</t>
-        </is>
-      </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>won</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Touches in penalty area</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Offsides</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Progressive runs</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Fouls suffered</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Through passes</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
-        <is>
-          <t>accurate through passes</t>
-        </is>
-      </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>xA</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>Second assists</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>Passes to final third</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
-        <is>
-          <t>accurate passes to final third</t>
-        </is>
-      </c>
-      <c r="BC1" t="inlineStr">
-        <is>
-          <t>Passes to penalty area / accurate</t>
-        </is>
-      </c>
-      <c r="BD1" t="inlineStr">
-        <is>
-          <t>Unnamed: 55</t>
-        </is>
-      </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>Passes to penalty area</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>Received passes</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>Forward passes</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
-        <is>
-          <t>accurate forward passes</t>
-        </is>
-      </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>Back passes</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
-        <is>
-          <t>accurate back passes</t>
-        </is>
-      </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>Conceded goals</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BK1" s="1" t="inlineStr">
         <is>
           <t>xCG</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BL1" s="1" t="inlineStr">
         <is>
           <t>Shots against</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
-        <is>
-          <t>Saves / with reflexes</t>
-        </is>
-      </c>
-      <c r="BN1" t="inlineStr">
-        <is>
-          <t>Unnamed: 65</t>
-        </is>
-      </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>Saves</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>with reflexes</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
         <is>
           <t>Exits</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
-        <is>
-          <t>Passes to GK / accurate</t>
-        </is>
-      </c>
-      <c r="BQ1" t="inlineStr">
-        <is>
-          <t>Unnamed: 68</t>
-        </is>
-      </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>Passes to GK</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
         <is>
           <t>Goal kicks</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BS1" s="1" t="inlineStr">
         <is>
           <t>Short goal kicks</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="BT1" s="1" t="inlineStr">
         <is>
           <t>Long goal kicks</t>
         </is>
@@ -4863,8 +4963,10 @@
           <t>England. League Two</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>46098</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5087,8 +5189,10 @@
           <t>England. League Two</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>46095</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -5311,8 +5415,10 @@
           <t>England. League Two</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>46088</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -5535,8 +5641,10 @@
           <t>England. League Two</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>46084</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -5759,8 +5867,10 @@
           <t>England. League Two</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>46081</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -5983,8 +6093,10 @@
           <t>England. League Two</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>46074</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -6207,8 +6319,10 @@
           <t>England. League Two</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
-        <v>46070</v>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -6431,8 +6545,10 @@
           <t>England. League Two</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
-        <v>46067</v>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
+        </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -6655,8 +6771,10 @@
           <t>England. League Two</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
-        <v>46060</v>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -6879,8 +6997,10 @@
           <t>England. League Two</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
-        <v>46053</v>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -7089,6 +7209,3734 @@
         <v>0</v>
       </c>
       <c r="BT11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:DB11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>match_name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>match_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>match_date</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>competition_name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>competition_id</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>season_name</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>season_id</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>competition_edition_id</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>minutes_full_all</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>count_match</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>count_match_failed</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>total_distance_full_all</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>total_metersperminute_full_all</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>running_distance_full_all</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>hsr_distance_full_all</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>hsr_count_full_all</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>sprint_distance_full_all</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>sprint_count_full_all</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>hi_distance_full_all</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>hi_count_full_all</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>psv99</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>psv99_top5</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>medaccel_count_full_all</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>highaccel_count_full_all</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>meddecel_count_full_all</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>highdecel_count_full_all</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>explacceltohsr_count_full_all</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>timetohsr_top3</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>timetohsrpostcod_top3</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>explacceltosprint_count_full_all</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>timetosprint_top3</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>timetosprintpostcod_top3</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>cod_count_full_all</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>timeto505around90_top3</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>timeto505around180_top3</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Match</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Minutes played</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Total actions</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>successful</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Goals</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>Assists</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Shots</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>on target</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>xG</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>Passes</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>Long passes</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Crosses</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>Dribbles</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>successful</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>Duels</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>won</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>Aerial duels</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>won</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>Interceptions</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>own half</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>Recoveries</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>opp. half</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>Yellow card</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>Red card</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>Defensive duels</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>won</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>Loose ball duels</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>won</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>Sliding tackles</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>successful</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>Clearances</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>Fouls</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>Yellow cards</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>Red cards</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>Shot assists</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>Offensive duels</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>won</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>Touches in penalty area</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>Offsides</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>Progressive runs</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>Fouls suffered</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>Through passes</t>
+        </is>
+      </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>xA</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>Second assists</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>Passes to final third</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>Passes to penalty area</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>Received passes</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>Forward passes</t>
+        </is>
+      </c>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="CP1" s="1" t="inlineStr">
+        <is>
+          <t>Back passes</t>
+        </is>
+      </c>
+      <c r="CQ1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>Conceded goals</t>
+        </is>
+      </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>xCG</t>
+        </is>
+      </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>Shots against</t>
+        </is>
+      </c>
+      <c r="CU1" s="1" t="inlineStr">
+        <is>
+          <t>Saves</t>
+        </is>
+      </c>
+      <c r="CV1" s="1" t="inlineStr">
+        <is>
+          <t>with reflexes</t>
+        </is>
+      </c>
+      <c r="CW1" s="1" t="inlineStr">
+        <is>
+          <t>Exits</t>
+        </is>
+      </c>
+      <c r="CX1" s="1" t="inlineStr">
+        <is>
+          <t>Passes to GK</t>
+        </is>
+      </c>
+      <c r="CY1" s="1" t="inlineStr">
+        <is>
+          <t>accurate</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>Goal kicks</t>
+        </is>
+      </c>
+      <c r="DA1" s="1" t="inlineStr">
+        <is>
+          <t>Short goal kicks</t>
+        </is>
+      </c>
+      <c r="DB1" s="1" t="inlineStr">
+        <is>
+          <t>Long goal kicks</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers FC v Harrogate Town FC</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2059160</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ENG - League Two</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>204</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>129</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I2" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="M2" t="n">
+        <v>116.11</v>
+      </c>
+      <c r="N2" t="n">
+        <v>1292</v>
+      </c>
+      <c r="O2" t="n">
+        <v>476</v>
+      </c>
+      <c r="P2" t="n">
+        <v>41</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>145</v>
+      </c>
+      <c r="R2" t="n">
+        <v>6</v>
+      </c>
+      <c r="S2" t="n">
+        <v>621</v>
+      </c>
+      <c r="T2" t="n">
+        <v>47</v>
+      </c>
+      <c r="U2" t="n">
+        <v>8.44</v>
+      </c>
+      <c r="V2" t="n">
+        <v>8.44</v>
+      </c>
+      <c r="W2" t="n">
+        <v>97</v>
+      </c>
+      <c r="X2" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>75</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="n">
+        <v>41</v>
+      </c>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers - Harrogate Town 0:3</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>England. League Two</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>LCMF, RWB</t>
+        </is>
+      </c>
+      <c r="AM2" t="n">
+        <v>68</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>42</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>21</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>18</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>13</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>17</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>7</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>5</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>9</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>5</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>3</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>7</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>2</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>2</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>2</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>12</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>9</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>5</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>2</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>2</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Fleetwood Town FC v Tranmere Rovers FC</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2058623</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ENG - League Two</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>204</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>129</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I3" t="n">
+        <v>21.47</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2312</v>
+      </c>
+      <c r="M3" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="N3" t="n">
+        <v>355</v>
+      </c>
+      <c r="O3" t="n">
+        <v>148</v>
+      </c>
+      <c r="P3" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>22</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>170</v>
+      </c>
+      <c r="T3" t="n">
+        <v>18</v>
+      </c>
+      <c r="U3" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="V3" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="W3" t="n">
+        <v>27</v>
+      </c>
+      <c r="X3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>19</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>2</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="n">
+        <v>11</v>
+      </c>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>Fleetwood Town - Tranmere Rovers 0:0</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>England. League Two</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>RCMF</t>
+        </is>
+      </c>
+      <c r="AM3" t="n">
+        <v>14</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CN3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers FC v Oldham Athletic AFC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2057600</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ENG - League Two</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>204</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>129</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I4" t="n">
+        <v>80.18000000000001</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>9001</v>
+      </c>
+      <c r="M4" t="n">
+        <v>112.26</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1345</v>
+      </c>
+      <c r="O4" t="n">
+        <v>660</v>
+      </c>
+      <c r="P4" t="n">
+        <v>63</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>221</v>
+      </c>
+      <c r="R4" t="n">
+        <v>13</v>
+      </c>
+      <c r="S4" t="n">
+        <v>881</v>
+      </c>
+      <c r="T4" t="n">
+        <v>76</v>
+      </c>
+      <c r="U4" t="n">
+        <v>8.640000000000001</v>
+      </c>
+      <c r="V4" t="n">
+        <v>8.640000000000001</v>
+      </c>
+      <c r="W4" t="n">
+        <v>113</v>
+      </c>
+      <c r="X4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>78</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>17</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="n">
+        <v>54</v>
+      </c>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers - Oldham Athletic 1:3</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>England. League Two</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="AM4" t="n">
+        <v>80</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>49</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>24</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>29</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>17</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>17</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>7</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>8</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>4</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>13</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>4</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX4" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY4" t="n">
+        <v>6</v>
+      </c>
+      <c r="BZ4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CA4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG4" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="CH4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CJ4" t="n">
+        <v>2</v>
+      </c>
+      <c r="CK4" t="n">
+        <v>3</v>
+      </c>
+      <c r="CL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM4" t="n">
+        <v>18</v>
+      </c>
+      <c r="CN4" t="n">
+        <v>8</v>
+      </c>
+      <c r="CO4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CP4" t="n">
+        <v>5</v>
+      </c>
+      <c r="CQ4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX4" t="n">
+        <v>2</v>
+      </c>
+      <c r="CY4" t="n">
+        <v>2</v>
+      </c>
+      <c r="CZ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Newport County AFC v Tranmere Rovers FC</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2057028</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ENG - League Two</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>204</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>129</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>Newport County - Tranmere Rovers 3:1</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>England. League Two</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>RB5, RW</t>
+        </is>
+      </c>
+      <c r="AM5" t="n">
+        <v>95</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>48</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>17</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>12</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>30</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>9</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>4</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>7</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>5</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>78</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>17</v>
+      </c>
+      <c r="BO5" t="n">
+        <v>6</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ5" t="n">
+        <v>2</v>
+      </c>
+      <c r="BR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BV5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY5" t="n">
+        <v>7</v>
+      </c>
+      <c r="BZ5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK5" t="n">
+        <v>3</v>
+      </c>
+      <c r="CL5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CM5" t="n">
+        <v>6</v>
+      </c>
+      <c r="CN5" t="n">
+        <v>7</v>
+      </c>
+      <c r="CO5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CP5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Crewe Alexandra FC v Tranmere Rovers FC</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2056670</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ENG - League Two</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>204</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>129</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I6" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>8608</v>
+      </c>
+      <c r="M6" t="n">
+        <v>137.73</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1577</v>
+      </c>
+      <c r="O6" t="n">
+        <v>713</v>
+      </c>
+      <c r="P6" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>183</v>
+      </c>
+      <c r="R6" t="n">
+        <v>10</v>
+      </c>
+      <c r="S6" t="n">
+        <v>896</v>
+      </c>
+      <c r="T6" t="n">
+        <v>70</v>
+      </c>
+      <c r="U6" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="V6" t="n">
+        <v>8.06</v>
+      </c>
+      <c r="W6" t="n">
+        <v>81</v>
+      </c>
+      <c r="X6" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>77</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>12</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="n">
+        <v>40</v>
+      </c>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>Crewe Alexandra - Tranmere Rovers 2:1</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>England. League Two</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>RWB</t>
+        </is>
+      </c>
+      <c r="AM6" t="n">
+        <v>62</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>45</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>14</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>14</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>9</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>19</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>8</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>11</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>6</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY6" t="n">
+        <v>4</v>
+      </c>
+      <c r="BZ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC6" t="n">
+        <v>2</v>
+      </c>
+      <c r="CD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI6" t="n">
+        <v>4</v>
+      </c>
+      <c r="CJ6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CK6" t="n">
+        <v>2</v>
+      </c>
+      <c r="CL6" t="n">
+        <v>2</v>
+      </c>
+      <c r="CM6" t="n">
+        <v>5</v>
+      </c>
+      <c r="CN6" t="n">
+        <v>7</v>
+      </c>
+      <c r="CO6" t="n">
+        <v>3</v>
+      </c>
+      <c r="CP6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CQ6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Notts County FC v Tranmere Rovers FC</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2055129</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ENG - League Two</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>204</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>129</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I7" t="n">
+        <v>53.53</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>6275</v>
+      </c>
+      <c r="M7" t="n">
+        <v>117.22</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1042</v>
+      </c>
+      <c r="O7" t="n">
+        <v>430</v>
+      </c>
+      <c r="P7" t="n">
+        <v>33</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>49</v>
+      </c>
+      <c r="R7" t="n">
+        <v>3</v>
+      </c>
+      <c r="S7" t="n">
+        <v>479</v>
+      </c>
+      <c r="T7" t="n">
+        <v>36</v>
+      </c>
+      <c r="U7" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="V7" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="W7" t="n">
+        <v>76</v>
+      </c>
+      <c r="X7" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>57</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>10</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="n">
+        <v>34</v>
+      </c>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>Notts County - Tranmere Rovers 5:0</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>England. League Two</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>RWB</t>
+        </is>
+      </c>
+      <c r="AM7" t="n">
+        <v>55</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>31</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>17</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>15</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>11</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>10</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>5</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>6</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY7" t="n">
+        <v>3</v>
+      </c>
+      <c r="BZ7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>2</v>
+      </c>
+      <c r="CE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>2</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM7" t="n">
+        <v>11</v>
+      </c>
+      <c r="CN7" t="n">
+        <v>3</v>
+      </c>
+      <c r="CO7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CP7" t="n">
+        <v>4</v>
+      </c>
+      <c r="CQ7" t="n">
+        <v>4</v>
+      </c>
+      <c r="CR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers FC v Accrington Stanley</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2054674</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-02-17</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ENG - League Two</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>204</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>129</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I8" t="n">
+        <v>99.58</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>11187</v>
+      </c>
+      <c r="M8" t="n">
+        <v>112.34</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1582</v>
+      </c>
+      <c r="O8" t="n">
+        <v>825</v>
+      </c>
+      <c r="P8" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>134</v>
+      </c>
+      <c r="R8" t="n">
+        <v>6</v>
+      </c>
+      <c r="S8" t="n">
+        <v>959</v>
+      </c>
+      <c r="T8" t="n">
+        <v>76</v>
+      </c>
+      <c r="U8" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="V8" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="W8" t="n">
+        <v>142</v>
+      </c>
+      <c r="X8" t="n">
+        <v>7</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>106</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr"/>
+      <c r="AD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="n">
+        <v>53</v>
+      </c>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers - Accrington Stanley 0:1</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>England. League Two</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>RB, RWB</t>
+        </is>
+      </c>
+      <c r="AM8" t="n">
+        <v>99</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>94</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>60</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>52</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>35</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>8</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>13</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>7</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>13</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>10</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>38</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>25</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>15</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>11</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>14</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>11</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>2</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BY8" t="n">
+        <v>17</v>
+      </c>
+      <c r="BZ8" t="n">
+        <v>11</v>
+      </c>
+      <c r="CA8" t="n">
+        <v>5</v>
+      </c>
+      <c r="CB8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>6</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>2</v>
+      </c>
+      <c r="CE8" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG8" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="CH8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI8" t="n">
+        <v>3</v>
+      </c>
+      <c r="CJ8" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK8" t="n">
+        <v>7</v>
+      </c>
+      <c r="CL8" t="n">
+        <v>5</v>
+      </c>
+      <c r="CM8" t="n">
+        <v>28</v>
+      </c>
+      <c r="CN8" t="n">
+        <v>21</v>
+      </c>
+      <c r="CO8" t="n">
+        <v>11</v>
+      </c>
+      <c r="CP8" t="n">
+        <v>10</v>
+      </c>
+      <c r="CQ8" t="n">
+        <v>10</v>
+      </c>
+      <c r="CR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW8" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX8" t="n">
+        <v>1</v>
+      </c>
+      <c r="CY8" t="n">
+        <v>1</v>
+      </c>
+      <c r="CZ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers FC v Crawley Town FC</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2054126</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ENG - League Two</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>204</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>129</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I9" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>11491</v>
+      </c>
+      <c r="M9" t="n">
+        <v>111.24</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1852</v>
+      </c>
+      <c r="O9" t="n">
+        <v>685</v>
+      </c>
+      <c r="P9" t="n">
+        <v>72</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>182</v>
+      </c>
+      <c r="R9" t="n">
+        <v>11</v>
+      </c>
+      <c r="S9" t="n">
+        <v>867</v>
+      </c>
+      <c r="T9" t="n">
+        <v>83</v>
+      </c>
+      <c r="U9" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="V9" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="W9" t="n">
+        <v>137</v>
+      </c>
+      <c r="X9" t="n">
+        <v>9</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>102</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>20</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>7</v>
+      </c>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="n">
+        <v>55</v>
+      </c>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers - Crawley Town 2:0</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>England. League Two</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>LWB, RWB</t>
+        </is>
+      </c>
+      <c r="AM9" t="n">
+        <v>103</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>51</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>21</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>23</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>12</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>20</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>9</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>9</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>6</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>7</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>15</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>8</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>11</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>56</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>5</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT9" t="n">
+        <v>2</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>2</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BW9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY9" t="n">
+        <v>4</v>
+      </c>
+      <c r="BZ9" t="n">
+        <v>2</v>
+      </c>
+      <c r="CA9" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE9" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI9" t="n">
+        <v>6</v>
+      </c>
+      <c r="CJ9" t="n">
+        <v>3</v>
+      </c>
+      <c r="CK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM9" t="n">
+        <v>10</v>
+      </c>
+      <c r="CN9" t="n">
+        <v>14</v>
+      </c>
+      <c r="CO9" t="n">
+        <v>6</v>
+      </c>
+      <c r="CP9" t="n">
+        <v>2</v>
+      </c>
+      <c r="CQ9" t="n">
+        <v>2</v>
+      </c>
+      <c r="CR9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA9" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Gillingham FC v Tranmere Rovers FC</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2052983</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ENG - League Two</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>204</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>129</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I10" t="n">
+        <v>73.47</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>8766</v>
+      </c>
+      <c r="M10" t="n">
+        <v>119.32</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1368</v>
+      </c>
+      <c r="O10" t="n">
+        <v>631</v>
+      </c>
+      <c r="P10" t="n">
+        <v>49</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>160</v>
+      </c>
+      <c r="R10" t="n">
+        <v>8</v>
+      </c>
+      <c r="S10" t="n">
+        <v>791</v>
+      </c>
+      <c r="T10" t="n">
+        <v>57</v>
+      </c>
+      <c r="U10" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="V10" t="n">
+        <v>8.33</v>
+      </c>
+      <c r="W10" t="n">
+        <v>92</v>
+      </c>
+      <c r="X10" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>68</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="n">
+        <v>38</v>
+      </c>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>Gillingham - Tranmere Rovers 2:1</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>England. League Two</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>RWB</t>
+        </is>
+      </c>
+      <c r="AM10" t="n">
+        <v>73</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>47</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>24</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>29</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>19</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>4</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>5</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>7</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>14</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>4</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>14</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX10" t="n">
+        <v>2</v>
+      </c>
+      <c r="BY10" t="n">
+        <v>10</v>
+      </c>
+      <c r="BZ10" t="n">
+        <v>3</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>3</v>
+      </c>
+      <c r="CB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>4</v>
+      </c>
+      <c r="CD10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG10" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="CH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI10" t="n">
+        <v>4</v>
+      </c>
+      <c r="CJ10" t="n">
+        <v>1</v>
+      </c>
+      <c r="CK10" t="n">
+        <v>3</v>
+      </c>
+      <c r="CL10" t="n">
+        <v>2</v>
+      </c>
+      <c r="CM10" t="n">
+        <v>20</v>
+      </c>
+      <c r="CN10" t="n">
+        <v>7</v>
+      </c>
+      <c r="CO10" t="n">
+        <v>2</v>
+      </c>
+      <c r="CP10" t="n">
+        <v>5</v>
+      </c>
+      <c r="CQ10" t="n">
+        <v>5</v>
+      </c>
+      <c r="CR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers FC v Salford City FC</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2051988</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ENG - League Two</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>204</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2025/2026</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>129</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1214</v>
+      </c>
+      <c r="I11" t="n">
+        <v>19.85</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2282</v>
+      </c>
+      <c r="M11" t="n">
+        <v>114.96</v>
+      </c>
+      <c r="N11" t="n">
+        <v>332</v>
+      </c>
+      <c r="O11" t="n">
+        <v>141</v>
+      </c>
+      <c r="P11" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>3</v>
+      </c>
+      <c r="R11" t="n">
+        <v>2</v>
+      </c>
+      <c r="S11" t="n">
+        <v>144</v>
+      </c>
+      <c r="T11" t="n">
+        <v>14</v>
+      </c>
+      <c r="U11" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="V11" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="W11" t="n">
+        <v>34</v>
+      </c>
+      <c r="X11" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>5</v>
+      </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="n">
+        <v>11</v>
+      </c>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>Tranmere Rovers - Salford City 0:2</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>England. League Two</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>RB</t>
+        </is>
+      </c>
+      <c r="AM11" t="n">
+        <v>20</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>11</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>8</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>6</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>5</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>4</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>5</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN11" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO11" t="n">
+        <v>2</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BV11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM11" t="n">
+        <v>7</v>
+      </c>
+      <c r="CN11" t="n">
+        <v>1</v>
+      </c>
+      <c r="CO11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CP11" t="n">
+        <v>2</v>
+      </c>
+      <c r="CQ11" t="n">
+        <v>2</v>
+      </c>
+      <c r="CR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY11" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB11" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>